<commit_message>
Sprint 9 Code review fixes
</commit_message>
<xml_diff>
--- a/Exc2/FURPS_table.xlsx
+++ b/Exc2/FURPS_table.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>Код</t>
   </si>
@@ -216,6 +216,12 @@
     <t xml:space="preserve">Совместимость необходима как из-за имеющихся тех. ограничений, так и из-за внутренней экспертизы</t>
   </si>
   <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>Масшатбируемость</t>
+  </si>
+  <si>
     <t>+R</t>
   </si>
   <si>
@@ -232,6 +238,12 @@
   </si>
   <si>
     <t xml:space="preserve">Макимальное использование имеющихся технологий (MS SQL и Oracle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Технологический стек ограничен Java, .NET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Для очереди сообщений может быть использована только Kafka</t>
   </si>
 </sst>
 </file>
@@ -286,7 +298,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="12">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -423,37 +435,11 @@
       </bottom>
       <diagonal style="none"/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -499,12 +485,6 @@
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="4" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="4" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
@@ -1272,78 +1252,102 @@
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="17"/>
+      <c r="D27" s="4"/>
     </row>
     <row r="28" ht="45">
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="29" ht="45">
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="14" t="s">
+    <row r="30" ht="30">
+      <c r="B30" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="17"/>
-    </row>
-    <row r="31" ht="35.25" customHeight="1">
-      <c r="A31" s="18"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="20" t="s">
+      <c r="D30" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D31" s="21"/>
+      <c r="C31" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="13"/>
     </row>
     <row r="32" ht="35.25" customHeight="1">
-      <c r="A32" s="18"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="D32" s="21"/>
+      <c r="A32" s="16"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="19"/>
     </row>
     <row r="33" ht="35.25" customHeight="1">
-      <c r="A33" s="18"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="D33" s="21"/>
-    </row>
-    <row r="34" ht="45">
-      <c r="A34" s="18"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="20" t="s">
+      <c r="A33" s="16"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D34" s="21"/>
-    </row>
-    <row r="35" ht="12.75"/>
+      <c r="D33" s="19"/>
+    </row>
+    <row r="34" ht="35.25" customHeight="1">
+      <c r="A34" s="16"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="19"/>
+    </row>
+    <row r="35" ht="45">
+      <c r="A35" s="16"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="19"/>
+    </row>
+    <row r="36" ht="30">
+      <c r="B36" s="17"/>
+      <c r="C36" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="19"/>
+    </row>
+    <row r="37" ht="30">
+      <c r="B37" s="17"/>
+      <c r="C37" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="19"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C4:D4"/>
@@ -1351,7 +1355,7 @@
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>

</xml_diff>